<commit_message>
Update Chef John to client-facing pricing and add Michelin premium framing
Replace chef cost prices with correct client prices across all four concepts (Tortilla/Pasta: $46→$38 volume, Grill & Grain: $50→$46 volume, Spice Route: $40 at 100-guest minimum). Update all add-on prices to client rates. Add Michelin-Trained premium callout in pricing summary. Update homepage and profile page to reflect new pricing and premium positioning.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/chef-menus/five-course-provisions/chef-john-menus-live.xlsx
+++ b/docs/chef-menus/five-course-provisions/chef-john-menus-live.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/doug/culinary-block-collective/docs/chef-menus/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/doug/culinary-block-collective/docs/chef-menus/five-course-provisions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{7E127C11-F240-5945-94E5-D80B94B4E4F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C8348746-667B-BA48-84CA-11083F748FCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1180" yWindow="1600" windowWidth="23500" windowHeight="15660" xr2:uid="{0DBC9A77-B31C-BC43-87FB-4D85EB9EBAB1}"/>
+    <workbookView xWindow="8740" yWindow="-17080" windowWidth="23500" windowHeight="15660" activeTab="2" xr2:uid="{0DBC9A77-B31C-BC43-87FB-4D85EB9EBAB1}"/>
   </bookViews>
   <sheets>
     <sheet name="The Tortilla Theory" sheetId="2" r:id="rId1"/>
@@ -1084,29 +1084,6 @@
   </si>
   <si>
     <t>main (veg)</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Pricing:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-50 guest minimum, $36/person</t>
-    </r>
   </si>
   <si>
     <r>
@@ -1513,6 +1490,30 @@
 choice of 2 burritos options OR
 choice of 2 sandwich options
 full condiment set</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Pricing:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+50 guest minimum, $36/person
+100 guest minimum, $32/person</t>
     </r>
   </si>
 </sst>
@@ -2412,13 +2413,13 @@
   <sheetData>
     <row r="1" spans="1:6" ht="119" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -2545,7 +2546,7 @@
         <v>69</v>
       </c>
       <c r="D10" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="E10" t="s">
         <v>70</v>
@@ -2774,7 +2775,7 @@
         <v>26</v>
       </c>
       <c r="B24" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C24" t="s">
         <v>49</v>
@@ -2944,13 +2945,13 @@
   <sheetData>
     <row r="1" spans="1:6" ht="136" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="3" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.2">
@@ -3528,7 +3529,7 @@
   <dimension ref="A1:F39"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="26" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.6640625" customWidth="1"/>
     <col min="2" max="2" width="28.83203125" customWidth="1"/>
     <col min="3" max="3" width="36.1640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9" bestFit="1" customWidth="1"/>
@@ -3538,13 +3539,13 @@
   <sheetData>
     <row r="1" spans="1:6" ht="102" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>351</v>
+        <v>369</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>356</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>357</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>358</v>
       </c>
     </row>
     <row r="3" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.2">
@@ -4151,13 +4152,13 @@
   <sheetData>
     <row r="1" spans="1:6" ht="85" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>359</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>360</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>361</v>
       </c>
     </row>
     <row r="3" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.2">
@@ -4216,7 +4217,7 @@
         <v>206</v>
       </c>
       <c r="C6" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="D6" t="s">
         <v>9</v>
@@ -4261,7 +4262,7 @@
         <v>63</v>
       </c>
       <c r="B9" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="C9" t="s">
         <v>250</v>
@@ -4578,7 +4579,7 @@
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="C28" t="s">
         <v>240</v>
@@ -4672,13 +4673,13 @@
   <sheetData>
     <row r="1" spans="1:6" ht="119" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>367</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>369</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>368</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">

</xml_diff>